<commit_message>
Mise à jour du tableau de synthèse + compétences BTS SIO
</commit_message>
<xml_diff>
--- a/Assets/Tbl-Synthèse.xlsx
+++ b/Assets/Tbl-Synthèse.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dasil\Desktop\Portfolio-HTML\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE9E92D-F6C3-4C5A-A3F4-CDBE95BB7CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6ACD0DD-B5DC-4B6A-A05F-D019D4BB0392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Print_Area_0" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$40</definedName>
-    <definedName name="Print_Area_0_0" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$40</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$40</definedName>
+    <definedName name="Print_Area_0" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$43</definedName>
+    <definedName name="Print_Area_0_0" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$43</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="69">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -86,11 +86,6 @@
 ▸Traiter des demandes concernant les applications</t>
   </si>
   <si>
-    <t>▸Participer à la valorisation de l’image de l’organisation sur les médias numériques en tenant compte du cadre juridique et des enjeux économiques
-▸Référencer les services en ligne de l’organisation et mesurer leur visibilité.
-▸Participer à l’évolution d’un site Web exploitant les données de l’organisation.</t>
-  </si>
-  <si>
     <t>▸Analyser les objectifs et les modalités d’organisation d’un projet
 ▸Planifier les activités
 ▸Évaluer les indicateurs de suivi d’un projet et analyser les écarts</t>
@@ -109,9 +104,6 @@
   <si>
     <t xml:space="preserve">Réalisation en cours de formation
 </t>
-  </si>
-  <si>
-    <t>Laboratoire de Préparation des Tests de Performances - Configuration LAMP</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
@@ -147,70 +139,10 @@
     <t>Centre de formation : H3 Campus Poissy</t>
   </si>
   <si>
-    <t>Labs Commandes de base système Linux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laboratoire d'Évaluation des Performances - Infrastructure Virtuelle pour l'Entreprise, (Calcul de RAM, mémoire, CPU…) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs Couche physique réseau </t>
-  </si>
-  <si>
-    <t>Lab -swicthing (filtrage, analyse de trames, test de connectivité..) Wireshark</t>
-  </si>
-  <si>
-    <t>toujours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dossiers de qualifications </t>
-  </si>
-  <si>
-    <t>mise en place d'écran de supervision Nommé Verdi (Dépèches)</t>
-  </si>
-  <si>
-    <t>Gestion de droits/ Gestion de l'AD (Ticketing de toute sorte)</t>
-  </si>
-  <si>
     <t>Adresse URL du portfolio : https://tms78.github.io/Portfolio-BTS/</t>
   </si>
   <si>
-    <t xml:space="preserve">Installation de machines virtuelles Linux ( Ubuntu et Kali) </t>
-  </si>
-  <si>
-    <t>Labs Arithmétique des ordinateurs et codage (binaire…)</t>
-  </si>
-  <si>
-    <t>Lab - Intro Scripts Shell/ Bash</t>
-  </si>
-  <si>
-    <t>Lab -Linux HA (Haute Availibility )</t>
-  </si>
-  <si>
-    <t>Lab -Veille technologique</t>
-  </si>
-  <si>
-    <t>Lab -Formation cyber ANSSI (Certification)</t>
-  </si>
-  <si>
-    <t>Lab -DATA-Integrity / cyber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs - Suivi Projet (HTTPS, DNS, DHCP…) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labs -Cyber (Attaque, firewall filtrage, chiffrement) </t>
-  </si>
-  <si>
     <t>1ère Année</t>
-  </si>
-  <si>
-    <t>Labs Infra Cisco ( vrai infra) / Inventaire INFRA</t>
-  </si>
-  <si>
-    <t>Labs réseau Packet Tracer : Configure IP, Switch, Router, Vlan, Routing, Cloisonement</t>
-  </si>
-  <si>
-    <t>Labs packet tracer - Protocols</t>
   </si>
   <si>
     <t>oct-25 / Nov-25</t>
@@ -228,21 +160,6 @@
     <t>Fevr-26 / Mars-26</t>
   </si>
   <si>
-    <t>Projet BTS</t>
-  </si>
-  <si>
-    <t>Gestion de droits/ Gestion de l'AD (Ticketing, assistance utilisateurs)</t>
-  </si>
-  <si>
-    <t>Gestion de parc (équipement)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dossiers de qualifications (Parc applicatif) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Migration machines vers NAGIOS anciennement PRTG </t>
-  </si>
-  <si>
     <t>Tout les 6mois</t>
   </si>
   <si>
@@ -255,16 +172,7 @@
     <t>nov-25 / 02-26</t>
   </si>
   <si>
-    <t>Sorti sur différents site : aide aux utilisateurs sur place</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monter de versions "SentinelOne" Antivirus, de nos machines projet (non-utilisateurs) </t>
-  </si>
-  <si>
     <t>mars-26 / mai-26</t>
-  </si>
-  <si>
-    <t>Configuration du superviseur Nagios ( Notifs, seuils, alertes, API…)</t>
   </si>
   <si>
     <t>N° candidat : 02543679666</t>
@@ -273,7 +181,99 @@
     <t>*</t>
   </si>
   <si>
-    <t>Sortis divers sur différents sites RATP (Accompagnements SI/ Support SI, Problème utilisateurs de NUIT, visite data center )</t>
+    <t>Mise en œuvre de mécanismes d’intégrité et de sécurité des données</t>
+  </si>
+  <si>
+    <t>Analyse de trames réseau et diagnostic de connectivité avec Wireshark</t>
+  </si>
+  <si>
+    <t>Déploiement d’une infrastructure web (stack LAMP)</t>
+  </si>
+  <si>
+    <t>Dimensionnement d’une infrastructure virtuelle (CPU, RAM, stockage)</t>
+  </si>
+  <si>
+    <t>Configuration d’une architecture réseau (adressage IP, VLAN, routage, cloisonnement) via Packet Tracer</t>
+  </si>
+  <si>
+    <t>Administration de base de systèmes Linux en ligne de commande</t>
+  </si>
+  <si>
+    <t>Déploiement et gestion de machines virtuelles Linux (Ubuntu, Kali)</t>
+  </si>
+  <si>
+    <t>Compréhension des fondamentaux du codage et de l’arithmétique binaire</t>
+  </si>
+  <si>
+    <t>Mise en place et gestion d’une infrastructure réseau (environnement Cisco réel)</t>
+  </si>
+  <si>
+    <t>Implémentation de solutions de haute disponibilité sous Linux</t>
+  </si>
+  <si>
+    <t>Analyse de la couche physique et des protocoles réseau</t>
+  </si>
+  <si>
+    <t>Étude et mise en œuvre des protocoles réseau via simulation (Packet Tracer)</t>
+  </si>
+  <si>
+    <t>Automatisation de tâches via scripts Shell / Bash</t>
+  </si>
+  <si>
+    <t>Réalisation d’une veille technologique dans le domaine informatique</t>
+  </si>
+  <si>
+    <t>Sensibilisation et formation aux bonnes pratiques en cybersécurité (référentiel ANSSI)</t>
+  </si>
+  <si>
+    <t>Mise en œuvre de mécanismes de cybersécurité (filtrage, chiffrement, firewall, tests d’attaque)</t>
+  </si>
+  <si>
+    <t>Déploiement et configuration de services réseau (HTTPS, DNS, DHCP)(Projet)</t>
+  </si>
+  <si>
+    <t>Conduite d’un projet informatique (Projet BTS)</t>
+  </si>
+  <si>
+    <t>Continuellement</t>
+  </si>
+  <si>
+    <t>Gestion des habilitations et des accès utilisateurs via Active Directory et outils internes (Droits réseau et admin…)</t>
+  </si>
+  <si>
+    <t>Traitement des incidents et demandes via outil de ticketing (support niveau 2)</t>
+  </si>
+  <si>
+    <t>Suivi et gestion du parc informatique (inventaire, conformité des équipements)</t>
+  </si>
+  <si>
+    <t>Optimisation du parc informatique (identification, retrait et réaffectation des équipements)</t>
+  </si>
+  <si>
+    <t>Réalisation de dossiers de qualification applicative pour dépoilement (parc logiciel)</t>
+  </si>
+  <si>
+    <t>Migration des équipements pour supervision de PRTG Network Monitor vers Nagios</t>
+  </si>
+  <si>
+    <t>Configuration du superviseur Nagios (seuils, alertes, notifications, API)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place d’écrans de supervision (affichage des alertes/dépèches en temps réel) Projet VERDI, GALAXIE </t>
+  </si>
+  <si>
+    <t>Déploiement de mise à jour de sécurité endpoint (SentinelOne) sur nos machines INFRA</t>
+  </si>
+  <si>
+    <t>Interventions techniques sur sites (support utilisateurs, accompagnement SI, visites data center)</t>
+  </si>
+  <si>
+    <t>Support technique de proximité sur site de nuit, pour les agents de nuit</t>
+  </si>
+  <si>
+    <t>▸Participer à la valorisation de l’image de l’organaisation sur les médias numériques en tenant compte du cadre juridique et des enjeux économiques
+▸Référencer les services en ligne de l’organisation et mesurer leur visibilité.
+▸Participer à l’évolution d’un site Web exploitant les données de l’organisation.</t>
   </si>
 </sst>
 </file>
@@ -337,11 +337,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
@@ -361,6 +356,12 @@
     <font>
       <b/>
       <sz val="22"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -626,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -649,70 +650,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="11" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="12" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1245,7 +1237,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AMK39"/>
+  <dimension ref="A1:AMK42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="65.06640625" style="1"/>
@@ -1256,18 +1248,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="36"/>
+      <c r="H1" s="33"/>
       <c r="AR1"/>
       <c r="AS1"/>
       <c r="AT1"/>
@@ -2251,16 +2243,16 @@
       <c r="AMJ1"/>
     </row>
     <row r="2" spans="1:1024" ht="41" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
       <c r="AR2"/>
       <c r="AS2"/>
       <c r="AT2"/>
@@ -3244,18 +3236,18 @@
       <c r="AMJ2"/>
     </row>
     <row r="3" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
+      <c r="A3" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
@@ -4242,18 +4234,18 @@
       <c r="AMJ3"/>
     </row>
     <row r="4" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="A4" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
       <c r="F4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>23</v>
+      <c r="G4" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>4</v>
@@ -5241,16 +5233,16 @@
       <c r="AMJ4"/>
     </row>
     <row r="5" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
+      <c r="A5" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
       <c r="AR5"/>
       <c r="AS5"/>
       <c r="AT5"/>
@@ -6234,10 +6226,10 @@
       <c r="AMJ5"/>
     </row>
     <row r="6" spans="1:1024" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="31" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -7241,8 +7233,8 @@
       <c r="AMJ6"/>
     </row>
     <row r="7" spans="1:1024" s="1" customFormat="1" ht="325.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="33"/>
-      <c r="B7" s="34"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="31"/>
       <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
@@ -7250,555 +7242,625 @@
         <v>14</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:1024" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
+      <c r="A8" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
     </row>
     <row r="9" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
+      <c r="A9" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
     </row>
     <row r="10" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="19">
+      <c r="A10" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="13">
         <v>45689</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="15"/>
+      <c r="C10" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="19">
+      <c r="A11" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="13">
         <v>45658</v>
       </c>
-      <c r="C11" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="15"/>
+      <c r="C11" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="19">
+      <c r="A12" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="13">
         <v>45658</v>
       </c>
-      <c r="C12" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="15"/>
+      <c r="C12" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="15"/>
+      <c r="A13" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="19">
+      <c r="A14" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="13">
         <v>45778</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="15"/>
+      <c r="C14" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="16"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" s="19">
+      <c r="A15" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="13">
         <v>45778</v>
       </c>
-      <c r="C15" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="15"/>
+      <c r="C15" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="16"/>
+      <c r="H15" s="10"/>
     </row>
     <row r="16" spans="1:1024" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="19">
+      <c r="A16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="13">
         <v>45717</v>
       </c>
-      <c r="C16" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="15"/>
+      <c r="C16" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="10"/>
     </row>
     <row r="17" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" s="19">
+      <c r="A17" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="13">
         <v>45901</v>
       </c>
-      <c r="C17" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="15"/>
+      <c r="C17" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G17" s="16"/>
+      <c r="H17" s="10"/>
     </row>
     <row r="18" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="19">
+      <c r="A18" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="13">
         <v>45962</v>
       </c>
-      <c r="C18" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H18" s="15"/>
+      <c r="C18" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="10"/>
     </row>
     <row r="19" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="19">
+      <c r="A19" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="13">
         <v>45962</v>
       </c>
-      <c r="C19" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="15"/>
+      <c r="C19" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" s="19">
+      <c r="A20" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="13">
         <v>45931</v>
       </c>
-      <c r="C20" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H20" s="15"/>
+      <c r="C20" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G22" s="25"/>
-      <c r="H22" s="15" t="s">
-        <v>67</v>
+      <c r="A22" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G22" s="16"/>
+      <c r="H22" s="10" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="19">
+      <c r="A23" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="13">
         <v>45597</v>
       </c>
-      <c r="C23" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="15" t="s">
-        <v>67</v>
+      <c r="C23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="10" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="17"/>
+      <c r="A24" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="11"/>
     </row>
     <row r="25" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C25" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="17"/>
+      <c r="A25" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G25" s="18"/>
+      <c r="H25" s="11"/>
     </row>
     <row r="26" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="G26" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="H26" s="17" t="s">
-        <v>67</v>
+      <c r="A26" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G26" s="18"/>
+      <c r="H26" s="11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="17.649999999999999" x14ac:dyDescent="0.35">
-      <c r="A27" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
+      <c r="A27" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
     </row>
     <row r="28" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="26"/>
+      <c r="A28" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="13" t="s">
+      <c r="A29" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G29" s="25"/>
-      <c r="H29" s="26"/>
+      <c r="B29" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
     </row>
     <row r="30" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B30" s="13" t="s">
+      <c r="A30" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H30" s="26"/>
+      <c r="B30" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
     </row>
     <row r="31" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B31" s="13">
-        <v>45691</v>
-      </c>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G31" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H31" s="26"/>
+      <c r="A31" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
     </row>
     <row r="32" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="14">
-        <v>45778</v>
-      </c>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H32" s="26"/>
+      <c r="C32" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
     </row>
     <row r="33" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="14">
-        <v>45717</v>
-      </c>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H33" s="26"/>
+      <c r="B33" s="24">
+        <v>45691</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H33" s="17" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="34" spans="1:8" ht="17.649999999999999" x14ac:dyDescent="0.35">
-      <c r="A34" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
+    <row r="34" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="25">
+        <v>45778</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H34" s="17"/>
     </row>
     <row r="35" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B35" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="10"/>
+      <c r="A35" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B35" s="25">
+        <v>45717</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="17"/>
     </row>
-    <row r="36" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C36" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G36" s="25"/>
-      <c r="H36" s="10"/>
+    <row r="36" spans="1:8" ht="17.649999999999999" x14ac:dyDescent="0.35">
+      <c r="A36" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
     </row>
     <row r="37" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H37" s="10"/>
+      <c r="A37" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="8"/>
     </row>
     <row r="38" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B38" s="24">
-        <v>45901</v>
-      </c>
-      <c r="C38" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D38" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E38" s="25"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="10"/>
+      <c r="A38" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="8"/>
     </row>
     <row r="39" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="8"/>
+    </row>
+    <row r="40" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="8"/>
+    </row>
+    <row r="41" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B39" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="G39" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H39" s="10"/>
+      <c r="B41" s="13">
+        <v>45901</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H41" s="8"/>
+    </row>
+    <row r="42" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -7808,7 +7870,7 @@
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A6:A7"/>

</xml_diff>